<commit_message>
Signature push anticipée + confirmation Live, feature GOTO Label/PREROLL avec saut réel synchronisé sur le vrai temps 1
</commit_message>
<xml_diff>
--- a/Viser.xlsx
+++ b/Viser.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tanaismusic/Documents/CLIC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{680896C3-F23E-E842-974E-86943AEC13F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B4F6ED4-B0C2-644B-A445-91DE9CBC32A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5180" yWindow="1800" windowWidth="28040" windowHeight="17440" xr2:uid="{2F1647A4-8C84-E14B-83BA-CB692A19D8A6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>MES</t>
   </si>
@@ -59,13 +59,25 @@
     <t>BREAK</t>
   </si>
   <si>
-    <t>REFRAIN</t>
-  </si>
-  <si>
     <t>COUPLET 1</t>
   </si>
   <si>
     <t>AD LIB</t>
+  </si>
+  <si>
+    <t>REFRAIN 2</t>
+  </si>
+  <si>
+    <t>REFRAIN 1</t>
+  </si>
+  <si>
+    <t>COUPLET 2</t>
+  </si>
+  <si>
+    <t>PONT</t>
+  </si>
+  <si>
+    <t>REFRAIN 3</t>
   </si>
 </sst>
 </file>
@@ -592,7 +604,7 @@
         <v>0</v>
       </c>
       <c r="D13" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
@@ -627,6 +639,9 @@
       <c r="C16">
         <v>0</v>
       </c>
+      <c r="D16" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17">
@@ -660,6 +675,9 @@
       <c r="C19">
         <v>0</v>
       </c>
+      <c r="D19" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20">
@@ -738,7 +756,7 @@
         <v>0</v>
       </c>
       <c r="D26" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
@@ -773,6 +791,9 @@
       <c r="C29">
         <v>0</v>
       </c>
+      <c r="D29" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30">
@@ -818,7 +839,7 @@
         <v>0</v>
       </c>
       <c r="D33" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
@@ -852,6 +873,9 @@
       </c>
       <c r="C36">
         <v>0</v>
+      </c>
+      <c r="D36" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Ajout mode Offline, module paroles (défilement + page web) et divers réglages
- Mode Offline : sélection d'un morceau (XLSX), PLAY/STOP, GOTO/PREROLL,
  simulation locale sans Live/MIDI, diffusion vers la page web 8765.
- lyrics.py : chargement des paroles (Lyrics/<morceau>.csv), correspondance
  mesure <-> ligne (8 mesures/ligne).
- Affichage défilant des paroles sur le grand écran (case à cocher dédiée,
  chiffres/points réduits de moitié et remontés en haut quand actif).
- Page web : boutons indépendants par appareil (paroles affichées/masquées,
  chiffres/points), diffusion du mode Offline.
- config.json : dots_only, offline_bpm, lyrics_enabled.
</commit_message>
<xml_diff>
--- a/Viser.xlsx
+++ b/Viser.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tanaismusic/Documents/CLIC/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/studiosvoa/Documents/CLIC-ABLETON-main/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B4F6ED4-B0C2-644B-A445-91DE9CBC32A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5E861B0-A55E-E64C-B96F-75AB67038C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5180" yWindow="1800" windowWidth="28040" windowHeight="17440" xr2:uid="{2F1647A4-8C84-E14B-83BA-CB692A19D8A6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>MES</t>
   </si>
@@ -56,13 +56,7 @@
     <t>INTRO</t>
   </si>
   <si>
-    <t>BREAK</t>
-  </si>
-  <si>
     <t>COUPLET 1</t>
-  </si>
-  <si>
-    <t>AD LIB</t>
   </si>
   <si>
     <t>REFRAIN 2</t>
@@ -78,6 +72,9 @@
   </si>
   <si>
     <t>REFRAIN 3</t>
+  </si>
+  <si>
+    <t>END</t>
   </si>
 </sst>
 </file>
@@ -518,7 +515,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -554,7 +551,7 @@
         <v>4</v>
       </c>
       <c r="C9">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -567,19 +564,19 @@
       <c r="C10">
         <v>0</v>
       </c>
+      <c r="D10" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C11">
-        <v>1</v>
-      </c>
-      <c r="D11" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
@@ -603,9 +600,6 @@
       <c r="C13">
         <v>0</v>
       </c>
-      <c r="D13" t="s">
-        <v>9</v>
-      </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14">
@@ -640,7 +634,7 @@
         <v>0</v>
       </c>
       <c r="D16" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
@@ -676,7 +670,7 @@
         <v>0</v>
       </c>
       <c r="D19" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
@@ -756,7 +750,7 @@
         <v>0</v>
       </c>
       <c r="D26" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
@@ -786,13 +780,13 @@
         <v>28</v>
       </c>
       <c r="B29">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C29">
         <v>0</v>
       </c>
       <c r="D29" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
@@ -800,7 +794,7 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C30">
         <v>0</v>
@@ -811,7 +805,7 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C31">
         <v>0</v>
@@ -822,7 +816,7 @@
         <v>31</v>
       </c>
       <c r="B32">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C32">
         <v>0</v>
@@ -833,13 +827,13 @@
         <v>32</v>
       </c>
       <c r="B33">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C33">
         <v>0</v>
       </c>
       <c r="D33" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
@@ -847,7 +841,7 @@
         <v>33</v>
       </c>
       <c r="B34">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C34">
         <v>0</v>
@@ -858,7 +852,7 @@
         <v>34</v>
       </c>
       <c r="B35">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C35">
         <v>0</v>
@@ -869,13 +863,13 @@
         <v>35</v>
       </c>
       <c r="B36">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C36">
         <v>0</v>
       </c>
       <c r="D36" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Feuilles de scène (xlsx) : ajout/mise à jour locale
</commit_message>
<xml_diff>
--- a/Viser.xlsx
+++ b/Viser.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tanaismusic/Documents/CLIC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B4F6ED4-B0C2-644B-A445-91DE9CBC32A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6B571EA-BB63-9245-89E6-3601A29E33DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5180" yWindow="1800" windowWidth="28040" windowHeight="17440" xr2:uid="{2F1647A4-8C84-E14B-83BA-CB692A19D8A6}"/>
+    <workbookView xWindow="4140" yWindow="1960" windowWidth="28040" windowHeight="17440" xr2:uid="{2F1647A4-8C84-E14B-83BA-CB692A19D8A6}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -56,13 +56,7 @@
     <t>INTRO</t>
   </si>
   <si>
-    <t>BREAK</t>
-  </si>
-  <si>
     <t>COUPLET 1</t>
-  </si>
-  <si>
-    <t>AD LIB</t>
   </si>
   <si>
     <t>REFRAIN 2</t>
@@ -71,13 +65,19 @@
     <t>REFRAIN 1</t>
   </si>
   <si>
-    <t>COUPLET 2</t>
-  </si>
-  <si>
     <t>PONT</t>
   </si>
   <si>
     <t>REFRAIN 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COUPLET 2 </t>
+  </si>
+  <si>
+    <t>FINAL</t>
+  </si>
+  <si>
+    <t>END</t>
   </si>
 </sst>
 </file>
@@ -518,10 +518,13 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C6">
         <v>0</v>
+      </c>
+      <c r="D6" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -573,13 +576,10 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C11">
-        <v>1</v>
-      </c>
-      <c r="D11" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
@@ -603,9 +603,6 @@
       <c r="C13">
         <v>0</v>
       </c>
-      <c r="D13" t="s">
-        <v>9</v>
-      </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14">
@@ -639,9 +636,6 @@
       <c r="C16">
         <v>0</v>
       </c>
-      <c r="D16" t="s">
-        <v>6</v>
-      </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17">
@@ -675,9 +669,6 @@
       <c r="C19">
         <v>0</v>
       </c>
-      <c r="D19" t="s">
-        <v>8</v>
-      </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20">
@@ -709,7 +700,7 @@
         <v>4</v>
       </c>
       <c r="C22">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
@@ -722,6 +713,9 @@
       <c r="C23">
         <v>0</v>
       </c>
+      <c r="D23" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24">
@@ -755,9 +749,6 @@
       <c r="C26">
         <v>0</v>
       </c>
-      <c r="D26" t="s">
-        <v>10</v>
-      </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27">
@@ -791,9 +782,6 @@
       <c r="C29">
         <v>0</v>
       </c>
-      <c r="D29" t="s">
-        <v>11</v>
-      </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30">
@@ -838,9 +826,6 @@
       <c r="C33">
         <v>0</v>
       </c>
-      <c r="D33" t="s">
-        <v>12</v>
-      </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34">
@@ -874,9 +859,6 @@
       <c r="C36">
         <v>0</v>
       </c>
-      <c r="D36" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37">
@@ -897,7 +879,7 @@
         <v>4</v>
       </c>
       <c r="C38">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
@@ -910,6 +892,9 @@
       <c r="C39">
         <v>0</v>
       </c>
+      <c r="D39" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40">
@@ -1007,10 +992,10 @@
         <v>4</v>
       </c>
       <c r="C48">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1020,8 +1005,11 @@
       <c r="C49">
         <v>0</v>
       </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D49" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>49</v>
       </c>
@@ -1032,7 +1020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>50</v>
       </c>
@@ -1043,7 +1031,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>51</v>
       </c>
@@ -1054,7 +1042,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>52</v>
       </c>
@@ -1065,7 +1053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>53</v>
       </c>
@@ -1076,7 +1064,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>54</v>
       </c>
@@ -1087,7 +1075,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>55</v>
       </c>
@@ -1098,7 +1086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>56</v>
       </c>
@@ -1109,7 +1097,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>57</v>
       </c>
@@ -1120,7 +1108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>58</v>
       </c>
@@ -1131,7 +1119,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>59</v>
       </c>
@@ -1142,7 +1130,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>60</v>
       </c>
@@ -1153,7 +1141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>61</v>
       </c>
@@ -1164,7 +1152,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>62</v>
       </c>
@@ -1175,7 +1163,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>63</v>
       </c>
@@ -1186,7 +1174,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>64</v>
       </c>
@@ -1196,8 +1184,11 @@
       <c r="C65">
         <v>0</v>
       </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D65" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>65</v>
       </c>
@@ -1208,7 +1199,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>66</v>
       </c>
@@ -1219,7 +1210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>67</v>
       </c>
@@ -1230,7 +1221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>68</v>
       </c>
@@ -1241,7 +1232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>69</v>
       </c>
@@ -1252,7 +1243,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>70</v>
       </c>
@@ -1263,7 +1254,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>71</v>
       </c>
@@ -1274,7 +1265,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>72</v>
       </c>
@@ -1285,7 +1276,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>73</v>
       </c>
@@ -1296,7 +1287,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>74</v>
       </c>
@@ -1307,7 +1298,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>75</v>
       </c>
@@ -1318,7 +1309,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>76</v>
       </c>
@@ -1329,7 +1320,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>77</v>
       </c>
@@ -1340,7 +1331,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>78</v>
       </c>
@@ -1351,7 +1342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>79</v>
       </c>
@@ -1359,10 +1350,10 @@
         <v>4</v>
       </c>
       <c r="C80">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>80</v>
       </c>
@@ -1372,8 +1363,11 @@
       <c r="C81">
         <v>0</v>
       </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>81</v>
       </c>
@@ -1384,7 +1378,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>82</v>
       </c>
@@ -1395,7 +1389,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>83</v>
       </c>
@@ -1406,7 +1400,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>84</v>
       </c>
@@ -1417,7 +1411,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>85</v>
       </c>
@@ -1428,7 +1422,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>86</v>
       </c>
@@ -1439,7 +1433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>87</v>
       </c>
@@ -1450,7 +1444,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>88</v>
       </c>
@@ -1461,7 +1455,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>89</v>
       </c>
@@ -1472,7 +1466,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>90</v>
       </c>
@@ -1483,7 +1477,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>91</v>
       </c>
@@ -1494,7 +1488,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>92</v>
       </c>
@@ -1505,7 +1499,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>93</v>
       </c>
@@ -1516,7 +1510,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>94</v>
       </c>
@@ -1527,7 +1521,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>95</v>
       </c>
@@ -1538,7 +1532,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>96</v>
       </c>
@@ -1548,8 +1542,11 @@
       <c r="C97">
         <v>0</v>
       </c>
-    </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D97" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>97</v>
       </c>
@@ -1560,7 +1557,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>98</v>
       </c>
@@ -1571,7 +1568,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>99</v>
       </c>
@@ -1582,7 +1579,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>100</v>
       </c>
@@ -1593,7 +1590,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>101</v>
       </c>
@@ -1604,7 +1601,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>102</v>
       </c>
@@ -1615,7 +1612,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>103</v>
       </c>
@@ -1626,7 +1623,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>104</v>
       </c>
@@ -1637,7 +1634,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A106">
         <v>105</v>
       </c>
@@ -1648,7 +1645,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A107">
         <v>106</v>
       </c>
@@ -1659,7 +1656,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A108">
         <v>107</v>
       </c>
@@ -1670,7 +1667,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A109">
         <v>108</v>
       </c>
@@ -1681,7 +1678,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A110">
         <v>109</v>
       </c>
@@ -1692,7 +1689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A111">
         <v>110</v>
       </c>
@@ -1703,7 +1700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A112">
         <v>111</v>
       </c>
@@ -1714,7 +1711,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A113">
         <v>112</v>
       </c>
@@ -1725,7 +1722,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A114">
         <v>113</v>
       </c>
@@ -1736,7 +1733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A115">
         <v>114</v>
       </c>
@@ -1747,7 +1744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A116">
         <v>115</v>
       </c>
@@ -1758,7 +1755,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A117">
         <v>116</v>
       </c>
@@ -1769,7 +1766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A118">
         <v>117</v>
       </c>
@@ -1780,7 +1777,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A119">
         <v>118</v>
       </c>
@@ -1791,7 +1788,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A120">
         <v>119</v>
       </c>
@@ -1802,7 +1799,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A121">
         <v>120</v>
       </c>
@@ -1813,7 +1810,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A122">
         <v>121</v>
       </c>
@@ -1824,7 +1821,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A123">
         <v>122</v>
       </c>
@@ -1835,7 +1832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A124">
         <v>123</v>
       </c>
@@ -1846,7 +1843,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A125">
         <v>124</v>
       </c>
@@ -1857,7 +1854,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A126">
         <v>125</v>
       </c>
@@ -1868,7 +1865,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A127">
         <v>126</v>
       </c>
@@ -1879,7 +1876,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A128">
         <v>127</v>
       </c>
@@ -1888,6 +1885,9 @@
       </c>
       <c r="C128">
         <v>0</v>
+      </c>
+      <c r="D128" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.2">

</xml_diff>